<commit_message>
feat(app): add per-account color family (account-colors.js)
Each account picks one of the 12 palette families, stored as data in
meta.account_style (D-2, DESIGN.md C8): checking defaults to tra,
savings to ali unless linked to a goal (D-impl-2, the hucha derives
its family from the goal) which gives imp, liability to coc.

account-colors.js reuses FAMILIES/isFamily from category-colors.js and
mirrors sanitizeStyleMap's defenses (__proto__, closed FAMILIES list).
goalFamily resolves a goal's family from its linked account.

schema.sql seeds account_style as '{}' (CONFIG-IN-META, no migration,
same precedent as quick_register); demo-ficticio.xlsx regenerated to
match. sw.js SHELL gains the new file.
</commit_message>
<xml_diff>
--- a/tests/app/fixtures/demo-ficticio.xlsx
+++ b/tests/app/fixtures/demo-ficticio.xlsx
@@ -405,7 +405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -527,9 +527,17 @@
         <v>{}</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>account_style</v>
+      </c>
+      <c r="B16" t="str">
+        <v>{}</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B16"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(app): add pay day preference and period start proposal logic
</commit_message>
<xml_diff>
--- a/tests/app/fixtures/demo-ficticio.xlsx
+++ b/tests/app/fixtures/demo-ficticio.xlsx
@@ -405,7 +405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -535,9 +535,17 @@
         <v>{}</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>pay_day</v>
+      </c>
+      <c r="B17" t="str">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B17"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>